<commit_message>
fixing the captured co2 problem
</commit_message>
<xml_diff>
--- a/data_5years.xlsx
+++ b/data_5years.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Paper - Nuclear DACSS\Code\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{668C59EF-7F06-45AA-A768-FEA54DCDBBA7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ABC8157A-134F-4618-8777-32DDF1EE6508}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
     <sheet name="co2_tax" sheetId="4" r:id="rId5"/>
     <sheet name="co2_storage_capacity" sheetId="5" r:id="rId6"/>
     <sheet name="nuclear_capex" sheetId="15" r:id="rId7"/>
-    <sheet name="uranium_prce" sheetId="19" r:id="rId8"/>
+    <sheet name="uranium_price" sheetId="19" r:id="rId8"/>
     <sheet name="capex" sheetId="6" r:id="rId9"/>
     <sheet name="electricity_emission_factor" sheetId="18" r:id="rId10"/>
     <sheet name="electricity_consumed" sheetId="17" r:id="rId11"/>

</xml_diff>